<commit_message>
chore: update ONE schedules 2026-08-05
</commit_message>
<xml_diff>
--- a/output/one_schedules_2026-08-05.xlsx
+++ b/output/one_schedules_2026-08-05.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,40 +446,50 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>POL</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ETD</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Vessel</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Voyage</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>ETD</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>POD</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>ETA</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>TransitDays</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Raw</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>ScrapedAt</t>
         </is>
@@ -501,24 +511,453 @@
           <t>SEGOT</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>(Parse pending)</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>ONE Solutions Support English HOME SCHEDULE PRICES BOOKING DOCUMENTATION MANAGE SHIPMENT FINANCE Search Schedule Search for schedules, book, and manage your shipment. User Guide Point to Point Vessel Port Long Range List Calendar POL/ POD Selection Go Green Origin Destination Date Next 2 Weeks Cargo</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2026-08-05 07:02 UTC</t>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>(Input error: Locator.click: Timeout 30000ms exceeded.
+Call log:
+waiting for locator("input").first.first
+  -   locator resolved to &lt;input id=":ri:" role="switch" type="checkbox" data-enabled="false" aria-labelledby=":ri:--label" class="mag-toggle__input mag-toggle__input--size-responsive mag-toggle__input--labelAlignment-left"/&gt;
+  - attempting click action
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #1
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #2
+  -   waiting 20ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #3
+  -   waiting 100ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #4
+  -   waiting 100ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #5
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #6
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #7
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #8
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #9
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #10
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #11
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #12
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #13
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #14
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #15
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #16
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #17
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #18
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #19
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #20
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #21
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #22
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #23
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #24
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #25
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #26
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #27
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #28
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #29
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #30
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #31
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #32
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #33
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #34
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #35
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #36
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #37
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #38
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #39
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #40
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #41
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #42
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #43
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #44
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #45
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #46
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #47
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #48
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #49
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #50
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #51
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #52
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #53
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #54
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #55
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #56
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #57
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #58
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #59
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #60
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #61
+  -   waiting 500ms
+)</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-08-05 07:16 UTC</t>
         </is>
       </c>
     </row>
@@ -538,24 +977,460 @@
           <t>NOOSL</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>(Parse pending)</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>ONE Solutions Support English HOME SCHEDULE PRICES BOOKING DOCUMENTATION MANAGE SHIPMENT FINANCE Search Schedule Search for schedules, book, and manage your shipment. User Guide Point to Point Vessel Port Long Range List Calendar POL/ POD Selection Go Green Origin HONG KONG, HONG KONG, CHINA (CY) De</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>2026-08-05 07:02 UTC</t>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>(Input error: Locator.click: Timeout 30000ms exceeded.
+Call log:
+waiting for locator("input").first.first
+  -   locator resolved to &lt;input id=":ri:" role="switch" type="checkbox" data-enabled="false" aria-labelledby=":ri:--label" class="mag-toggle__input mag-toggle__input--size-responsive mag-toggle__input--labelAlignment-left"/&gt;
+  - attempting click action
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #1
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #2
+  -   waiting 20ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #3
+  -   waiting 100ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #4
+  -   waiting 100ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #5
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #6
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #7
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #8
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #9
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #10
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #11
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #12
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #13
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #14
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #15
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #16
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #17
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #18
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #19
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #20
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #21
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #22
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #23
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #24
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #25
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #26
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #27
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #28
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #29
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #30
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #31
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #32
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #33
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #34
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #35
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #36
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #37
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #38
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #39
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #40
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #41
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #42
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #43
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #44
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #45
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #46
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #47
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #48
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #49
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #50
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #51
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #52
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #53
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #54
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #55
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #56
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #57
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #58
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #59
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #60
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #61
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #62
+  -   waiting 500ms
+)</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-08-05 07:17 UTC</t>
         </is>
       </c>
     </row>
@@ -575,24 +1450,933 @@
           <t>NOTAE</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>(Parse pending)</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>ONE Solutions Support English HOME SCHEDULE PRICES BOOKING DOCUMENTATION MANAGE SHIPMENT FINANCE Search Schedule Search for schedules, book, and manage your shipment. User Guide Point to Point Vessel Port Long Range List Calendar POL/ POD Selection Go Green Origin HO CHI MINH, VIETNAM (CY) TANANGER,</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>2026-08-05 07:02 UTC</t>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>(Input error: Locator.click: Timeout 30000ms exceeded.
+Call log:
+waiting for locator("input").first.first
+  -   locator resolved to &lt;input id=":ri:" role="switch" type="checkbox" data-enabled="false" aria-labelledby=":ri:--label" class="mag-toggle__input mag-toggle__input--size-responsive mag-toggle__input--labelAlignment-left"/&gt;
+  - attempting click action
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #1
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #2
+  -   waiting 20ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #3
+  -   waiting 100ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #4
+  -   waiting 100ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #5
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #6
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #7
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #8
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #9
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #10
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #11
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #12
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #13
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #14
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #15
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #16
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #17
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #18
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #19
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #20
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #21
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #22
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #23
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #24
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #25
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #26
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #27
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #28
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #29
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #30
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #31
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #32
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #33
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #34
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #35
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #36
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #37
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #38
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #39
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #40
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #41
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #42
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #43
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #44
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #45
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #46
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #47
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #48
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #49
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #50
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #51
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #52
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #53
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #54
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #55
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #56
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #57
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #58
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #59
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #60
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #61
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #62
+  -   waiting 500ms
+)</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-08-05 07:18 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CNTAO→ITSPE</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CNTAO</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ITSPE</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>(Input error: Locator.click: Timeout 30000ms exceeded.
+Call log:
+waiting for locator("input").first.first
+  -   locator resolved to &lt;input id=":ri:" role="switch" type="checkbox" data-enabled="false" aria-labelledby=":ri:--label" class="mag-toggle__input mag-toggle__input--size-responsive mag-toggle__input--labelAlignment-left"/&gt;
+  - attempting click action
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #1
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #2
+  -   waiting 20ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #3
+  -   waiting 100ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #4
+  -   waiting 100ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #5
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #6
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #7
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #8
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #9
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #10
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #11
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #12
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #13
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #14
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #15
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #16
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #17
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #18
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #19
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #20
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #21
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #22
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #23
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #24
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #25
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #26
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #27
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #28
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #29
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #30
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #31
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #32
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #33
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #34
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #35
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #36
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #37
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #38
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #39
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #40
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #41
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #42
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #43
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #44
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #45
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #46
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #47
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #48
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #49
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #50
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #51
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #52
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #53
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #54
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #55
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #56
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #57
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #58
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #59
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #60
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #61
+  -   waiting 500ms
+  -   waiting for element to be visible, enabled and stable
+  -   element is visible, enabled and stable
+  -   scrolling into view if needed
+  -   done scrolling
+  -   &lt;label for=":ri:" id=":ri:--root" class="mag-toggle__base mag-toggle__base--size-responsive mag-toggle__base--labelAlignment-left"&gt;…&lt;/label&gt; intercepts pointer events
+  - retrying click action, attempt #62
+  -   waiting 500ms
+)</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-08-05 07:18 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>